<commit_message>
Nettoyer le suivi intervenants et aligner sur les scripts montés
Recadrer T11/E20/E21, synchroniser les transcripts Video*.docx, filtrer les fiches sur les affectations finales, et ne garder que les derniers mails/guides à envoyer tout en conservant les réponses.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/20260723_Prev_Vid.xlsx
+++ b/data/20260723_Prev_Vid.xlsx
@@ -1105,18 +1105,18 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Muriel : peur du manque de temps, de l’échec et de la perte de légitimité ; nécessité de réorganiser ses responsabilités. Jean-Jacques : impossibilité de tout maîtriser, risque d’échec et nécessité d’accepter l’incertitude. Loïc : caractère clivant de l’entrepreneuriat dans le milieu académique et ajustement du discours. Sylvia : urgence d’aller jusqu’au patient, difficultés de financement et accomplissement personnel. La fin rassemble leurs conseils les plus forts.</t>
+          <t>Muriel : expérience enrichissante, « intégrateur social », impact visible de la recherche. Loïc : comité scientifique tout en gardant ses fonctions d'enseignant-chercheur ; impartialité. Jean-Jacques : conseil de surveillance — engagement sous une autre forme. Fil monté : ce que ça change dans le métier ; ce qu'il faut concilier.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>E20 — Gérer les freins. Temps, légitimité, entourage, droit à l’apprentissage et sécurisation du parcours. 
-E21 — Innover comme processus d’apprentissage. Incertitude, essais, erreurs, pivot et progression plutôt que réussite linéaire. (focaliser le discours sur les leviers existant pour vaincre les freins)</t>
+          <t>E20 — Concilier recherche et engagement dans l'innovation. Double casquette, gouvernance, impartialité, évolution du métier de chercheur. 
+E21 — Gérer les freins et innover comme apprentissage. Temps, légitimité, entourage, doute ; incertitude, essais, pivot ; première action réversible.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>L’apprenant identifie ses propres freins et comprend qu’ils ne doivent pas tous être résolus avant de faire le premier pas. Il choisit une première action réaliste et réversible.</t>
+          <t>L'apprenant comprend comment l'innovation transforme le métier de chercheur : casquettes multiples, conciliation des responsabilités, impact visible — sans opposer recherche et engagement.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>L’apprenant sait préparer une première collaboration en clarifiant les contributions, les attentes, les règles de décision et les sujets de propriété intellectuelle.</t>
+          <t>L'apprenant sait identifier les dispositifs d'accompagnement utiles et préparer une première collaboration en clarifiant contributions, attentes et sujets de propriété intellectuelle.</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1214,13 +1214,13 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>À constituer à partir des sélections Clarisse « Passer à l’action » (conseils, idées reçues à déconstruire, message final).</t>
+          <t>Chorale conclusion : se lancer malgré les doutes, ne pas attendre la certitude, solidarité des entrepreneurs, petits pas, formation utile même sans créer d'entreprise.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>L’apprenant repart avec un premier pas concret et un message clair pour oser engager une démarche d’innovation.</t>
+          <t>L'apprenant repart avec un premier pas concret et un message clair pour oser engager une démarche d'innovation (doutes, solidarité, petits pas).</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Ajouter le script E7 de Stephanie Sano et un retour unique E6+E7.
Les Word envoyés reprennent ses textes inchangés, avec les remarques en orange à la première personne.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/20260723_Prev_Vid.xlsx
+++ b/data/20260723_Prev_Vid.xlsx
@@ -710,8 +710,8 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>E6 — Le réflexe de déclaration avant toute divulgation. Confidentialité, nouveauté, publication, congrès, soutenance et DI. 
-E7 — À qui parler et avec quoi arriver ? Premier contact, rôle du chargé de valorisation et informations utiles pour examiner un résultat.</t>
+          <t>E6 — Stephanie Sano : Le réflexe de déclaration avant toute divulgation. Confidentialité, nouveauté, publication, congrès, soutenance et DI. 
+E7 — Stephanie Sano : À qui parler et avec quoi arriver ? Premier contact, rôle du chargé de valorisation et informations utiles pour examiner un résultat.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1150,7 +1150,7 @@
       <c r="E22" s="5" t="inlineStr">
         <is>
           <t>E22 — Pascal Corbel : Concevoir une collaboration équilibrée. Objectifs partagés, complémentarité, gouvernance, engagement, création et partage de valeur. 
-E23 — Antoine Latreille : Sécuriser juridiquement la collaboration. Confidentialité, contrats, connaissances antérieures, résultats nouveaux, PI, publication et sortie du partenariat.</t>
+E23 — Eneli Vino : Sécuriser juridiquement la collaboration. Confidentialité, contrats, connaissances antérieures, résultats nouveaux, PI, publication et sortie du partenariat.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Ajouter les revues 1 des scripts E8 et E9 de Stanislas De Lapasse.
Dépose les scripts reçus, annote le cadrage pédagogique (chorale T5, grain E8/E9), aligne l’intervenant retenu et régénère le site.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/20260723_Prev_Vid.xlsx
+++ b/data/20260723_Prev_Vid.xlsx
@@ -781,8 +781,8 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>E8 — Choisir un mode de protection adapté. Brevetabilité, secret, savoir-faire, logiciel, preuve et confidentialité. 
-E9 — La PI comme actif stratégique. Barrière à l’entrée, pouvoir de négociation, crédibilité et articulation avec le modèle de valorisation.</t>
+          <t>E8 — Stanislas De Lapasse : Choisir un mode de protection adapté. Brevetabilité, secret, savoir-faire, logiciel, preuve et confidentialité. 
+E9 — Stanislas De Lapasse : La PI comme actif stratégique. Barrière à l’entrée, pouvoir de négociation, crédibilité et articulation avec le modèle de valorisation.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">

</xml_diff>